<commit_message>
Fix exemple YoY marge : (D-C)*100 pour les points (marge stockee en fraction)
La marge est une fraction (0,166), donc =D-C vaut 0,0065 et le format '0,0 pt'
affichait '0,0'. Correction : =(D6-C6)*100 = 0,65 -> '+ 0,6 pt'. Note explicative
mise a jour.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EXEMPLES_COCKPIT.xlsx
+++ b/eduservices/EXEMPLES_COCKPIT.xlsx
@@ -1101,18 +1101,18 @@
         <v/>
       </c>
       <c r="E6" s="19">
-        <f>D6-C6</f>
+        <f>(D6-C6)*100</f>
         <v/>
       </c>
       <c r="F6" s="20">
-        <f>D6-C6   ← EN POINTS (16,6% − 16,0% = +0,6 pt)</f>
+        <f>(D6-C6)*100   ← ×100 car la marge est une FRACTION (0,166) → +0,6 pt</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Pourquoi : une marge est déjà un %. Sa variation « en % » (16,6/16,0−1 = +4,0 %) est trompeuse — on croit +4 points. La bonne lecture = la DIFFÉRENCE de points : 16,6 % − 16,0 % = +0,6 pt. Formule : =D6-C6, format personnalisé "+ "0.0" pt".</t>
+          <t>Pourquoi : une marge est déjà un %. Sa variation « en % » (16,6/16,0−1 = +4,0 %) est trompeuse — on croit +4 points. La bonne lecture = la DIFFÉRENCE de points : 16,6 % − 16,0 % = +0,6 pt. ATTENTION : la marge est stockée en FRACTION (0,166), donc =D6-C6 vaut 0,0065 → le format afficherait « 0,0 pt ». Il faut ×100 : =(D6-C6)*100 = 0,65 → format "+ "0.0" pt" → + 0,6 pt.</t>
         </is>
       </c>
     </row>

</xml_diff>